<commit_message>
Added images and videos
</commit_message>
<xml_diff>
--- a/src/Hollow Knight Silksong Boss Rankings.xlsx
+++ b/src/Hollow Knight Silksong Boss Rankings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CJ\Documents\My Projects\hollow-knight-silksong-boss-ranking\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC8FD363-6620-45B4-816E-E731D768B297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EFE406F-7016-4774-83F6-862438A8B934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="117">
   <si>
     <t>ID</t>
   </si>
@@ -261,6 +261,138 @@
   </si>
   <si>
     <t>Image</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=P5CsSXCPbCzA9GCD</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=P5CsSXCPbCzA9GCD&amp;t=60</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=P5CsSXCPbCzA9GCD&amp;t=186</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=P5CsSXCPbCzA9GCD&amp;t=348</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=P5CsSXCPbCzA9GCD&amp;t=510</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=P5CsSXCPbCzA9GCD&amp;t=648</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=P5CsSXCPbCzA9GCD&amp;t=803</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=P5CsSXCPbCzA9GCD&amp;t=1008</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=1245</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=1380</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=1500</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=1770</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=2306</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=2070</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=2689</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=3116</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=3220</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=3498</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=3630</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=3752</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=3995</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=4210</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=4673</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=4874</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=5010</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=5175</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=5366</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=5828</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=6000</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=6180</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=6325</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=5QJqIaSBqcRvJnoa&amp;t=6416</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=6494</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=6558</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=6795</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=7055</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=7173</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=7240</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=7386</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=7635</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=7797</t>
+  </si>
+  <si>
+    <t>https://youtu.be/00rXa-VboV8?si=dRTc5nt0FjzaxIXg&amp;t=7930</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Av6b4_BKXlM?si=BR28F0rmy5n_Nfu-</t>
+  </si>
+  <si>
+    <t>Skarsinger Karmelita</t>
   </si>
 </sst>
 </file>
@@ -270,10 +402,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -296,10 +436,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -307,8 +448,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="19">
@@ -2445,7 +2588,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{49CEFBDD-59FE-4C2D-8E7D-C1B76BE0AF72}" name="QualityTable" displayName="QualityTable" ref="A1:R46" totalsRowShown="0">
   <autoFilter ref="A1:R46" xr:uid="{49CEFBDD-59FE-4C2D-8E7D-C1B76BE0AF72}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R46">
-    <sortCondition ref="K1:K46"/>
+    <sortCondition ref="B1:B46"/>
   </sortState>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{513B421C-E20A-4CE1-BB11-439F161A4329}" name="ID">
@@ -2454,7 +2597,7 @@
     <tableColumn id="3" xr3:uid="{41544CA9-AB72-4557-B30B-486E0159305B}" name="Boss"/>
     <tableColumn id="11" xr3:uid="{41426B42-369C-40E7-B7C2-E38250FB5D84}" name="Act"/>
     <tableColumn id="16" xr3:uid="{4AE7E68E-DAB6-485E-9E28-8A0CB2650DE4}" name="Image" dataDxfId="0">
-      <calculatedColumnFormula>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</calculatedColumnFormula>
+      <calculatedColumnFormula>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{A953B013-1BCC-465F-B101-DD7C4B4A3463}" name="Video"/>
     <tableColumn id="2" xr3:uid="{43DF05CD-EC58-4594-91FA-FD87DF786F47}" name="Raime" dataDxfId="17"/>
@@ -2858,6 +3001,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="25.6640625" customWidth="1"/>
+    <col min="4" max="4" width="8.88671875" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="11" max="11" width="10.21875" customWidth="1"/>
     <col min="12" max="12" width="14.88671875" customWidth="1"/>
@@ -2923,116 +3067,122 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2">
-        <f t="shared" ref="A2:A46" si="0">ROW()-1</f>
+        <f>ROW()-1</f>
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Skarsinger_Kamelita.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Bell_Beast.png</v>
+      </c>
+      <c r="E2" t="s">
+        <v>74</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="K2">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>2</v>
+        <v>27.2</v>
       </c>
       <c r="L2">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>1.3</v>
+        <v>-0.3</v>
       </c>
       <c r="M2">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="N2">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="O2">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="P2">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>0.63</v>
+        <v>2.79</v>
       </c>
       <c r="Q2" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="R2" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="C3">
         <v>3</v>
       </c>
       <c r="D3" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Lost_Lace.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Bell_Eater.png</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>97</v>
       </c>
       <c r="F3">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="K3">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>2.4</v>
+        <v>22.6</v>
       </c>
       <c r="L3">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-1.8</v>
+        <v>-0.8</v>
       </c>
       <c r="M3">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="N3">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="O3">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P3">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
@@ -3040,373 +3190,376 @@
       </c>
       <c r="Q3" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="R3" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/First_Sinner.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Broodmother.png</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>96</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="I4">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="J4">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="K4">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>2.4</v>
+        <v>31.6</v>
       </c>
       <c r="L4">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-0.5</v>
+        <v>3</v>
       </c>
       <c r="M4">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="N4">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="O4">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="P4">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>0.8</v>
+        <v>6.44</v>
       </c>
       <c r="Q4" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="R4" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Cogwork_Dancers.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Clover_Dancers.png</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G5">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I5">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="J5">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="K5">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>6</v>
+        <v>13.4</v>
       </c>
       <c r="L5">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>1.3</v>
+        <v>0.8</v>
       </c>
       <c r="M5">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="N5">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O5">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="P5">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>0.89</v>
+        <v>5.78</v>
       </c>
       <c r="Q5" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R5" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Last_Judge.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Cogwork_Dancers.png</v>
+      </c>
+      <c r="E6" t="s">
+        <v>84</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G6">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K6">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>7.4</v>
+        <v>6</v>
       </c>
       <c r="L6">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-4.3</v>
+        <v>1.3</v>
       </c>
       <c r="M6">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="N6">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O6">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="P6">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>5.24</v>
+        <v>0.89</v>
       </c>
       <c r="Q6" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Lace_2.png</v>
-      </c>
-      <c r="F7">
-        <v>14</v>
-      </c>
-      <c r="G7">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <v>5</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Craggler.png</v>
       </c>
       <c r="I7">
-        <v>8</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="K7">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="L7">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-3.8</v>
+        <v>-42</v>
       </c>
       <c r="M7">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="N7">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="O7">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="P7">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.29</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="R7" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D8" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Widow.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Crawfather.png</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>113</v>
       </c>
       <c r="F8">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G8">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="J8">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="K8">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>8</v>
+        <v>22.4</v>
       </c>
       <c r="L8">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-2.5</v>
+        <v>-3</v>
       </c>
       <c r="M8">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="N8">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O8">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="P8">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.76</v>
+        <v>6.22</v>
       </c>
       <c r="Q8" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="R8" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Grand_Mother_Silk.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Crust_King_Khann.png</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>102</v>
       </c>
       <c r="F9">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="H9">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I9">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="J9">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="K9">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>8.1999999999999993</v>
+        <v>15.8</v>
       </c>
       <c r="L9">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-0.3</v>
+        <v>1.5</v>
       </c>
       <c r="M9">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="N9">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O9">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
@@ -3414,370 +3567,388 @@
       </c>
       <c r="P9">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.25</v>
+        <v>3.31</v>
       </c>
       <c r="Q9" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R9" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10" t="str">
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Disgraced_Chef_Luigoli.png</v>
+      </c>
+      <c r="E10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F10">
+        <v>25</v>
+      </c>
+      <c r="G10">
+        <v>25</v>
+      </c>
+      <c r="H10">
+        <v>28</v>
+      </c>
+      <c r="I10">
+        <v>36</v>
+      </c>
+      <c r="J10">
         <v>35</v>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Tormented_Trobbio.png</v>
-      </c>
-      <c r="F10">
-        <v>11</v>
-      </c>
-      <c r="G10">
-        <v>7</v>
-      </c>
-      <c r="H10">
-        <v>9</v>
-      </c>
-      <c r="I10">
-        <v>5</v>
-      </c>
-      <c r="J10">
-        <v>9</v>
       </c>
       <c r="K10">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>8.1999999999999993</v>
+        <v>29.8</v>
       </c>
       <c r="L10">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>1</v>
+        <v>6.5</v>
       </c>
       <c r="M10">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="N10">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="O10">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="P10">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.04</v>
+        <v>4.79</v>
       </c>
       <c r="Q10" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="R10" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="C11">
         <v>2</v>
       </c>
       <c r="D11" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Second_Sentinel.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Father_of_the_Flame.png</v>
+      </c>
+      <c r="E11" t="s">
+        <v>90</v>
       </c>
       <c r="F11">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="H11">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="I11">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="J11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="K11">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>10.25</v>
+        <v>34.75</v>
       </c>
       <c r="L11">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>2.2999999999999998</v>
+        <v>-5</v>
       </c>
       <c r="M11">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="N11">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="O11">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P11">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.49</v>
+        <v>3.9</v>
       </c>
       <c r="Q11" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="R11" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
       <c r="D12" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Trobbio.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/First_Sinner.png</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>94</v>
       </c>
       <c r="F12">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H12">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I12">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K12">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>10.8</v>
+        <v>2.4</v>
       </c>
       <c r="L12">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="M12">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="N12">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O12">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="P12">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.64</v>
+        <v>0.8</v>
       </c>
       <c r="Q12" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Phantom.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Forebrothers_Signis_and_Gron.png</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
       </c>
       <c r="F13">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="G13">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="H13">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I13">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="J13">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="K13">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>12.4</v>
+        <v>23.2</v>
       </c>
       <c r="L13">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>3.3</v>
+        <v>-2.8</v>
       </c>
       <c r="M13">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="N13">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="O13">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="P13">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>1.62</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="Q13" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="R13" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Shrine_Guardian_Seth.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Fourth_Chorus.png</v>
+      </c>
+      <c r="E14" t="s">
+        <v>76</v>
       </c>
       <c r="F14">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G14">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="I14">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J14">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="K14">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>13.2</v>
+        <v>19.2</v>
       </c>
       <c r="L14">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-2.8</v>
+        <v>8.5</v>
       </c>
       <c r="M14">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="N14">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="O14">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="P14">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>8.3800000000000008</v>
+        <v>5.34</v>
       </c>
       <c r="Q14" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R14" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D15" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Clover_Dancers.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Grand_Mother_Silk.png</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="F15">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G15">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I15">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="J15">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="K15">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>13.4</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="L15">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>0.8</v>
+        <v>-0.3</v>
       </c>
       <c r="M15">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="N15">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
@@ -3785,572 +3956,602 @@
       </c>
       <c r="O15">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="P15">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>5.78</v>
+        <v>3.25</v>
       </c>
       <c r="Q15" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R15" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Shakra.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Great_Conchflies.png</v>
+      </c>
+      <c r="E16" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16">
+        <v>22</v>
       </c>
       <c r="G16">
-        <v>20</v>
+        <v>33</v>
+      </c>
+      <c r="H16">
+        <v>21</v>
       </c>
       <c r="I16">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="J16">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="K16">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>15</v>
+        <v>27.8</v>
       </c>
       <c r="L16">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-3</v>
+        <v>0.3</v>
       </c>
       <c r="M16">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="N16">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="O16">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="P16">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.56</v>
+        <v>5.64</v>
       </c>
       <c r="Q16" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R16" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17" t="str">
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Groal_the_Great.png</v>
+      </c>
+      <c r="E17" t="s">
+        <v>93</v>
+      </c>
+      <c r="F17">
+        <v>37</v>
+      </c>
+      <c r="G17">
         <v>26</v>
       </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Lace_1.png</v>
-      </c>
-      <c r="F17">
-        <v>20</v>
-      </c>
-      <c r="G17">
-        <v>16</v>
-      </c>
       <c r="H17">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="I17">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="J17">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="K17">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>15.8</v>
+        <v>36.4</v>
       </c>
       <c r="L17">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>0.3</v>
+        <v>4.5</v>
       </c>
       <c r="M17">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="N17">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="O17">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="P17">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.4</v>
+        <v>5.31</v>
       </c>
       <c r="Q17" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="R17" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="C18">
         <v>3</v>
       </c>
       <c r="D18" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Crust_King_Khann.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Gurr_the_Outcast.png</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>103</v>
       </c>
       <c r="F18">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="G18">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H18">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="I18">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J18">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="K18">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>15.8</v>
+        <v>32.4</v>
       </c>
       <c r="L18">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>1.5</v>
+        <v>5.8</v>
       </c>
       <c r="M18">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="N18">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="O18">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="P18">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.31</v>
+        <v>5.28</v>
       </c>
       <c r="Q18" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="R18" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
       <c r="D19" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Fourth_Chorus.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Lace_1.png</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="F19">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G19">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H19">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="I19">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J19">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="K19">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>19.2</v>
+        <v>15.8</v>
       </c>
       <c r="L19">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>8.5</v>
+        <v>0.3</v>
       </c>
       <c r="M19">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="N19">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O19">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="P19">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>5.34</v>
+        <v>2.4</v>
       </c>
       <c r="Q19" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R19" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Raging_Conchfly.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Lace_2.png</v>
+      </c>
+      <c r="E20" t="s">
+        <v>85</v>
       </c>
       <c r="F20">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G20">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="H20">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I20">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="J20">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="K20">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>19.600000000000001</v>
+        <v>8</v>
       </c>
       <c r="L20">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>4.3</v>
+        <v>-3.8</v>
       </c>
       <c r="M20">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="N20">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="O20">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="P20">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>8.57</v>
+        <v>3.29</v>
       </c>
       <c r="Q20" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R20" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
       <c r="D21" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Sister_Splinter.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Last_Judge.png</v>
+      </c>
+      <c r="E21" t="s">
+        <v>83</v>
       </c>
       <c r="F21">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="G21">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="H21">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I21">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="J21">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="K21">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>19.8</v>
+        <v>7.4</v>
       </c>
       <c r="L21">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-2.2999999999999998</v>
+        <v>-4.3</v>
       </c>
       <c r="M21">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="N21">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="O21">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P21">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>5.46</v>
+        <v>5.24</v>
       </c>
       <c r="Q21" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R21" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Moorwing.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Lost_Garmond.png</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>104</v>
       </c>
       <c r="F22">
-        <v>18</v>
-      </c>
-      <c r="G22">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="H22">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I22">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J22">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="K22">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>20.6</v>
+        <v>23.25</v>
       </c>
       <c r="L22">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-2</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="M22">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="N22">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="O22">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="P22">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.38</v>
+        <v>6.1</v>
       </c>
       <c r="Q22" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R22" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="C23">
         <v>3</v>
       </c>
       <c r="D23" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Crawfather.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Lost_Lace.png</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>114</v>
       </c>
       <c r="F23">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="G23">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="I23">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="K23">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>22.4</v>
+        <v>2.4</v>
       </c>
       <c r="L23">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-3</v>
+        <v>-1.8</v>
       </c>
       <c r="M23">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="N23">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="O23">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="P23">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>6.22</v>
+        <v>2.33</v>
       </c>
       <c r="Q23" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R23" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D24" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Bell_Eater.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Moorwing.png</v>
+      </c>
+      <c r="E24" t="s">
+        <v>77</v>
       </c>
       <c r="F24">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G24">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H24">
+        <v>18</v>
+      </c>
+      <c r="I24">
+        <v>27</v>
+      </c>
+      <c r="J24">
         <v>19</v>
-      </c>
-      <c r="I24">
-        <v>26</v>
-      </c>
-      <c r="J24">
-        <v>22</v>
       </c>
       <c r="K24">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="L24">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-0.8</v>
+        <v>-2</v>
       </c>
       <c r="M24">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N24">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O24">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P24">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.33</v>
+        <v>3.38</v>
       </c>
       <c r="Q24" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
@@ -4363,541 +4564,568 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="C25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Nyleth.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Moss_Mother.png</v>
+      </c>
+      <c r="E25" t="s">
+        <v>73</v>
       </c>
       <c r="F25">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="G25">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="H25">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="I25">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="J25">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="K25">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="L25">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>8.8000000000000007</v>
+        <v>2.5</v>
       </c>
       <c r="M25">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="N25">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="O25">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="P25">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>4.5999999999999996</v>
+        <v>2.1</v>
       </c>
       <c r="Q25" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R25" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Forebrothers_Signis_and_Gron.png</v>
-      </c>
-      <c r="F26">
-        <v>28</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Moss_Mother_Duo.png</v>
+      </c>
+      <c r="E26" t="s">
+        <v>81</v>
       </c>
       <c r="G26">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="H26">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I26">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="J26">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="K26">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>23.2</v>
+        <v>29.25</v>
       </c>
       <c r="L26">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-2.8</v>
+        <v>-0.3</v>
       </c>
       <c r="M26">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="N26">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="O26">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P26">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>4.3499999999999996</v>
+        <v>4.0199999999999996</v>
       </c>
       <c r="Q26" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="R26" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C27">
         <v>3</v>
       </c>
       <c r="D27" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Lost_Garmond.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Nyleth.png</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>101</v>
       </c>
       <c r="F27">
-        <v>13</v>
+        <v>21</v>
+      </c>
+      <c r="G27">
+        <v>23</v>
       </c>
       <c r="H27">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I27">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="J27">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="K27">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>23.25</v>
+        <v>23</v>
       </c>
       <c r="L27">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>2.2999999999999998</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="M27">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N27">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="O27">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P27">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>6.1</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="Q27" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="R27" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C28">
         <v>3</v>
       </c>
       <c r="D28" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Watcher_at_thhe_Edge.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Pale_Stag.png</v>
+      </c>
+      <c r="E28" t="s">
+        <v>105</v>
       </c>
       <c r="F28">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="H28">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I28">
-        <v>23</v>
+        <v>43</v>
+      </c>
+      <c r="J28">
+        <v>38</v>
       </c>
       <c r="K28">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>26</v>
+        <v>39.25</v>
       </c>
       <c r="L28">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-26</v>
+        <v>-1.7</v>
       </c>
       <c r="M28">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="N28">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="O28">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="P28">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.4500000000000002</v>
+        <v>3.56</v>
       </c>
       <c r="Q28" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R28" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29" t="str">
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Phantom.png</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F29">
+        <v>12</v>
+      </c>
+      <c r="G29">
+        <v>13</v>
+      </c>
+      <c r="H29">
+        <v>12</v>
+      </c>
+      <c r="I29">
+        <v>10</v>
+      </c>
+      <c r="J29">
         <v>15</v>
-      </c>
-      <c r="C29">
-        <v>2</v>
-      </c>
-      <c r="D29" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/The_Unraveled.png</v>
-      </c>
-      <c r="F29">
-        <v>31</v>
-      </c>
-      <c r="G29">
-        <v>32</v>
-      </c>
-      <c r="H29">
-        <v>30</v>
-      </c>
-      <c r="I29">
-        <v>19</v>
-      </c>
-      <c r="J29">
-        <v>24</v>
       </c>
       <c r="K29">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>27.2</v>
+        <v>12.4</v>
       </c>
       <c r="L29">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-4</v>
+        <v>3.3</v>
       </c>
       <c r="M29">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="N29">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="O29">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="P29">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>4.96</v>
+        <v>1.62</v>
       </c>
       <c r="Q29" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="R29" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C30">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Bell_Beast.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Pinstress.png</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>98</v>
       </c>
       <c r="F30">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G30">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="H30">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="I30">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="J30">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="K30">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>27.2</v>
+        <v>28</v>
       </c>
       <c r="L30">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-0.3</v>
+        <v>5</v>
       </c>
       <c r="M30">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="N30">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O30">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="P30">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.79</v>
+        <v>5.4</v>
       </c>
       <c r="Q30" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R30" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Great_Conchflies.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Plasmified_Zago.png</v>
+      </c>
+      <c r="E31" t="s">
+        <v>112</v>
       </c>
       <c r="F31">
-        <v>22</v>
-      </c>
-      <c r="G31">
+        <v>40</v>
+      </c>
+      <c r="H31">
+        <v>39</v>
+      </c>
+      <c r="I31">
         <v>33</v>
-      </c>
-      <c r="H31">
-        <v>21</v>
-      </c>
-      <c r="I31">
-        <v>35</v>
-      </c>
-      <c r="J31">
-        <v>28</v>
       </c>
       <c r="K31">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>27.8</v>
+        <v>37.333333333333336</v>
       </c>
       <c r="L31">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>0.3</v>
+        <v>-37.299999999999997</v>
       </c>
       <c r="M31">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="N31">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="O31">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="P31">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>5.64</v>
+        <v>3.09</v>
       </c>
       <c r="Q31" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="R31" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32" t="str">
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Raging_Conchfly.png</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F32">
         <v>19</v>
       </c>
-      <c r="C32">
-        <v>3</v>
-      </c>
-      <c r="D32" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Pinstress.png</v>
-      </c>
-      <c r="F32">
-        <v>27</v>
-      </c>
       <c r="G32">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H32">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="I32">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="J32">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="K32">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>28</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="L32">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="M32">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="N32">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="O32">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="P32">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>5.4</v>
+        <v>8.57</v>
       </c>
       <c r="Q32" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="R32" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A33">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
       <c r="D33" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Moss_Mother_Duo.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Savage_Beastfly.png</v>
+      </c>
+      <c r="E33" t="s">
+        <v>88</v>
+      </c>
+      <c r="F33">
+        <v>41</v>
       </c>
       <c r="G33">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H33">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="I33">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J33">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K33">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>29.25</v>
+        <v>35.6</v>
       </c>
       <c r="L33">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-0.3</v>
+        <v>-3.3</v>
       </c>
       <c r="M33">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="N33">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="O33">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
@@ -4905,364 +5133,382 @@
       </c>
       <c r="P33">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>4.0199999999999996</v>
+        <v>3.83</v>
       </c>
       <c r="Q33" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="R33" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C34">
         <v>2</v>
       </c>
       <c r="D34" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Disgraced_Chef_Luigoli.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Second_Sentinel.png</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>110</v>
       </c>
       <c r="F34">
-        <v>25</v>
-      </c>
-      <c r="G34">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H34">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="I34">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="J34">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="K34">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>29.8</v>
+        <v>10.25</v>
       </c>
       <c r="L34">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>6.5</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="M34">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="N34">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="O34">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="P34">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>4.79</v>
+        <v>3.49</v>
       </c>
       <c r="Q34" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R34" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="C35">
         <v>2</v>
       </c>
       <c r="D35" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Broodmother.png</v>
-      </c>
-      <c r="F35">
-        <v>33</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Shakra.png</v>
+      </c>
+      <c r="E35" t="s">
+        <v>115</v>
       </c>
       <c r="G35">
-        <v>19</v>
-      </c>
-      <c r="H35">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="I35">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="J35">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="K35">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>31.6</v>
+        <v>15</v>
       </c>
       <c r="L35">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="M35">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="N35">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="O35">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="P35">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>6.44</v>
+        <v>3.56</v>
       </c>
       <c r="Q35" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="R35" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Voltvyrm.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Shrine_Guardian_Seth.png</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>100</v>
       </c>
       <c r="F36">
-        <v>23</v>
+        <v>4</v>
+      </c>
+      <c r="G36">
+        <v>29</v>
       </c>
       <c r="H36">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="I36">
-        <v>40</v>
+        <v>12</v>
+      </c>
+      <c r="J36">
+        <v>11</v>
       </c>
       <c r="K36">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>32</v>
+        <v>13.2</v>
       </c>
       <c r="L36">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-32</v>
+        <v>-2.8</v>
       </c>
       <c r="M36">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="N36">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="O36">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="P36">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>6.98</v>
+        <v>8.3800000000000008</v>
       </c>
       <c r="Q36" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="R36" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Gurr_the_Outcast.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Sister_Splinter.png</v>
+      </c>
+      <c r="E37" t="s">
+        <v>78</v>
       </c>
       <c r="F37">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="G37">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H37">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="I37">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="J37">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="K37">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>32.4</v>
+        <v>19.8</v>
       </c>
       <c r="L37">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>5.8</v>
+        <v>-2.2999999999999998</v>
       </c>
       <c r="M37">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="N37">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="O37">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="P37">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>5.28</v>
+        <v>5.46</v>
       </c>
       <c r="Q37" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="R37" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="C38">
+        <v>3</v>
+      </c>
+      <c r="D38" t="str">
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Skarsinger_Karmelita.png</v>
+      </c>
+      <c r="E38" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>2</v>
+      </c>
+      <c r="H38">
         <v>1</v>
       </c>
-      <c r="D38" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Moss_Mother.png</v>
-      </c>
-      <c r="F38">
-        <v>36</v>
-      </c>
-      <c r="G38">
-        <v>35</v>
-      </c>
-      <c r="H38">
-        <v>31</v>
-      </c>
       <c r="I38">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="J38">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="K38">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="L38">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="M38">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="N38">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="O38">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P38">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.1</v>
+        <v>0.63</v>
       </c>
       <c r="Q38" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="R38" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A39">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Father_of_the_Flame.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Skull_Tyrant.png</v>
+      </c>
+      <c r="E39" t="s">
+        <v>80</v>
       </c>
       <c r="F39">
-        <v>35</v>
+        <v>34</v>
+      </c>
+      <c r="G39">
+        <v>31</v>
       </c>
       <c r="H39">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="I39">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="J39">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="K39">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>34.75</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="L39">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-5</v>
+        <v>4</v>
       </c>
       <c r="M39">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="N39">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
@@ -5270,249 +5516,252 @@
       </c>
       <c r="O39">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P39">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.9</v>
+        <v>2.93</v>
       </c>
       <c r="Q39" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R39" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C40">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D40" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Savage_Beastfly.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Summoned_Savior.png</v>
       </c>
       <c r="F40">
-        <v>41</v>
-      </c>
-      <c r="G40">
-        <v>36</v>
-      </c>
-      <c r="H40">
         <v>38</v>
-      </c>
-      <c r="I40">
-        <v>30</v>
-      </c>
-      <c r="J40">
-        <v>33</v>
       </c>
       <c r="K40">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>35.6</v>
+        <v>38</v>
       </c>
       <c r="L40">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-3.3</v>
+        <v>-38</v>
       </c>
       <c r="M40">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="N40">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="O40">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="P40">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.83</v>
+        <v>0</v>
       </c>
       <c r="Q40" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R40" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A41">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Skull_Tyrant.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/The_Unraveled.png</v>
+      </c>
+      <c r="E41" t="s">
+        <v>107</v>
       </c>
       <c r="F41">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G41">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H41">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="I41">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="J41">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="K41">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>35.799999999999997</v>
+        <v>27.2</v>
       </c>
       <c r="L41">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>4</v>
+        <v>-4</v>
       </c>
       <c r="M41">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="N41">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="O41">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="P41">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>2.93</v>
+        <v>4.96</v>
       </c>
       <c r="Q41" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="R41" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>35</v>
+      </c>
+      <c r="C42">
+        <v>3</v>
+      </c>
+      <c r="D42" t="str">
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Tormented_Trobbio.png</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F42">
+        <v>11</v>
+      </c>
+      <c r="G42">
+        <v>7</v>
+      </c>
+      <c r="H42">
         <v>9</v>
       </c>
-      <c r="C42">
-        <v>2</v>
-      </c>
-      <c r="D42" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Groal_the_Great.png</v>
-      </c>
-      <c r="F42">
-        <v>37</v>
-      </c>
-      <c r="G42">
-        <v>26</v>
-      </c>
-      <c r="H42">
-        <v>40</v>
-      </c>
       <c r="I42">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J42">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="K42">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>36.4</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="L42">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="M42">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="N42">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="O42">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="P42">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>5.31</v>
+        <v>2.04</v>
       </c>
       <c r="Q42" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="R42" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="C43">
         <v>2</v>
       </c>
       <c r="D43" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Plasmified_Zago.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Trobbio.png</v>
+      </c>
+      <c r="E43" t="s">
+        <v>86</v>
       </c>
       <c r="F43">
-        <v>40</v>
+        <v>16</v>
+      </c>
+      <c r="G43">
+        <v>10</v>
       </c>
       <c r="H43">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="I43">
-        <v>33</v>
+        <v>9</v>
+      </c>
+      <c r="J43">
+        <v>10</v>
       </c>
       <c r="K43">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>37.333333333333336</v>
+        <v>10.8</v>
       </c>
       <c r="L43">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-37.299999999999997</v>
+        <v>-1</v>
       </c>
       <c r="M43">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="N43">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="O43">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
@@ -5520,183 +5769,229 @@
       </c>
       <c r="P43">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.09</v>
+        <v>2.64</v>
       </c>
       <c r="Q43" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="R43" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="C44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D44" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Summoned_Savior.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Voltvyrm.png</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="F44">
-        <v>38</v>
+        <v>23</v>
+      </c>
+      <c r="H44">
+        <v>33</v>
+      </c>
+      <c r="I44">
+        <v>40</v>
       </c>
       <c r="K44">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="L44">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-38</v>
+        <v>-32</v>
       </c>
       <c r="M44">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="N44">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="O44">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="P44">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>0</v>
+        <v>6.98</v>
       </c>
       <c r="Q44" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="R44" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A45">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="C45">
         <v>3</v>
       </c>
       <c r="D45" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Pale_Stag.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Watcher_at_thhe_Edge.png</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>108</v>
       </c>
       <c r="F45">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="H45">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="I45">
-        <v>43</v>
-      </c>
-      <c r="J45">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="K45">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>39.25</v>
+        <v>26</v>
       </c>
       <c r="L45">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-1.7</v>
+        <v>-26</v>
       </c>
       <c r="M45">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="N45">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="O45">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="P45">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>3.56</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="Q45" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="R45" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C46">
         <v>1</v>
       </c>
       <c r="D46" t="str">
-        <f>"../Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
-        <v>../Boss_Images/Craggler.png</v>
+        <f>"/Boss_Images/"&amp;SUBSTITUTE(QualityTable[[#This Row],[Boss]]," ","_")&amp;".png"</f>
+        <v>/Boss_Images/Widow.png</v>
+      </c>
+      <c r="E46" t="s">
+        <v>79</v>
+      </c>
+      <c r="F46">
+        <v>9</v>
+      </c>
+      <c r="G46">
+        <v>6</v>
+      </c>
+      <c r="H46">
+        <v>6</v>
       </c>
       <c r="I46">
-        <v>42</v>
+        <v>13</v>
+      </c>
+      <c r="J46">
+        <v>6</v>
       </c>
       <c r="K46">
         <f>AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="L46">
         <f>ROUND(QualityTable[[#This Row],[Me]]-AVERAGE(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Ratheil]]),1)</f>
-        <v>-42</v>
+        <v>-2.5</v>
       </c>
       <c r="M46">
         <f>MAX(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="N46">
         <f>MIN(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]])</f>
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="O46">
         <f>QualityTable[[#This Row],[Max]]-QualityTable[[#This Row],[Min]]</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P46">
         <f>ROUND(_xlfn.STDEV.P(QualityTable[[#This Row],[Raime]]:QualityTable[[#This Row],[Me]]),2)</f>
-        <v>0</v>
+        <v>2.76</v>
       </c>
       <c r="Q46" s="4">
         <f>COUNTIFS(QualityTable[Average],"&lt;="&amp;QualityTable[[#This Row],[Average]],QualityTable[Act],QualityTable[[#This Row],[Act]])</f>
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="R46" s="4">
         <f>_xlfn.MAXIFS(QualityTable[Act_Rank],QualityTable[Act],QualityTable[[#This Row],[Act]])-QualityTable[[#This Row],[Act_Rank]]</f>
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E19" r:id="rId1" xr:uid="{915F70B4-0819-4EFF-8B23-D0BB342658BC}"/>
+    <hyperlink ref="E15" r:id="rId2" xr:uid="{843DEE0F-EC85-498A-A2FC-CD672C976B1B}"/>
+    <hyperlink ref="E29" r:id="rId3" xr:uid="{91523825-6F62-4A29-8FA0-B254AA543A01}"/>
+    <hyperlink ref="E12" r:id="rId4" xr:uid="{A28FAD2C-BD28-4456-A751-9068B8F360F9}"/>
+    <hyperlink ref="E32" r:id="rId5" xr:uid="{8F7AD108-82A9-4A97-A63C-129BBC3454C9}"/>
+    <hyperlink ref="E4" r:id="rId6" xr:uid="{6BFA06A3-9AE5-466A-B5BB-28AB1EE873B9}"/>
+    <hyperlink ref="E3" r:id="rId7" xr:uid="{3C86F1EC-7C50-441A-B7DE-AF91D7DD29A0}"/>
+    <hyperlink ref="E30" r:id="rId8" xr:uid="{3D24867E-58AE-4B98-8B6C-5A9A568CB5B3}"/>
+    <hyperlink ref="E36" r:id="rId9" xr:uid="{F3C9DEF2-8693-41CA-A750-E6FF955C4A1A}"/>
+    <hyperlink ref="E27" r:id="rId10" xr:uid="{6EF7E9C0-6F50-4E6E-B676-16AE5D016765}"/>
+    <hyperlink ref="E9" r:id="rId11" xr:uid="{D43288FB-4C6C-4B46-B12A-6D9D1D9C0082}"/>
+    <hyperlink ref="E18" r:id="rId12" xr:uid="{9535AB97-B08C-4AA3-A67E-D3C7BFA86B96}"/>
+    <hyperlink ref="E22" r:id="rId13" xr:uid="{563B90E6-BA36-41BC-AEB5-B3D9D9742CF2}"/>
+    <hyperlink ref="E5" r:id="rId14" xr:uid="{E5C5DD3F-7D21-439C-87FD-17E8F5710C0F}"/>
+    <hyperlink ref="E45" r:id="rId15" xr:uid="{1765720B-E451-41C1-8C75-EB7B5546AB7D}"/>
+    <hyperlink ref="E44" r:id="rId16" xr:uid="{3DD50295-E57C-4F91-8B83-A0C0F5A52AF1}"/>
+    <hyperlink ref="E34" r:id="rId17" xr:uid="{37985CBE-98CD-49C3-B570-4C3CCBC08E91}"/>
+    <hyperlink ref="E42" r:id="rId18" xr:uid="{5F3925DA-D73F-416D-9979-3077D70D3853}"/>
+    <hyperlink ref="E8" r:id="rId19" xr:uid="{C41640A1-C287-4DF8-BDCF-876EDD2BF39C}"/>
+    <hyperlink ref="E23" r:id="rId20" xr:uid="{D8CCDC49-3663-4C5D-AEE4-A48E10707394}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId21"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>